<commit_message>
Updated HGT pipeline doc
</commit_message>
<xml_diff>
--- a/data/putative_HGT-inserts/Putative-HGT_counts.xlsx
+++ b/data/putative_HGT-inserts/Putative-HGT_counts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/Documents/Zhuzhi genomes/HGT/HGT_pipeline/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/Documents/Zhuzhi genomes/HGT/HGT_pipeline/data/putative_HGT-inserts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E4F1DEB-8ACA-1A45-BAE8-BF4460DDAA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7140E14-02D7-1249-8883-C12A0C5CB107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3300" yWindow="2780" windowWidth="41600" windowHeight="23220" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>Genome</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Macropanesthia lithgowae</t>
   </si>
   <si>
-    <t>Periplaneta americana</t>
-  </si>
-  <si>
     <t>Blattella germanica</t>
   </si>
   <si>
@@ -117,6 +114,12 @@
   </si>
   <si>
     <t>Number of duplicate HGT inserts removed</t>
+  </si>
+  <si>
+    <t>Periplaneta americana v1</t>
+  </si>
+  <si>
+    <t>Name/Source</t>
   </si>
 </sst>
 </file>
@@ -209,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -223,6 +226,7 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -557,357 +561,371 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40A815C-EDAC-574C-BA26-EF35C495DFC6}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" customWidth="1"/>
-    <col min="5" max="5" width="26.5" customWidth="1"/>
-    <col min="6" max="6" width="54.33203125" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="29.33203125" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="22.5" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" customWidth="1"/>
+    <col min="6" max="6" width="26.5" customWidth="1"/>
+    <col min="7" max="7" width="54.33203125" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+    <col min="9" max="9" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="9"/>
+      <c r="C2" s="2">
         <v>3425</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>200.9970802919708</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>3006</v>
       </c>
-      <c r="E2" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F2" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="9"/>
+      <c r="C3" s="2">
         <v>1196</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="2">
         <v>189.12959866220737</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3" s="2">
         <v>14815</v>
       </c>
-      <c r="E3" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F3" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="9"/>
+      <c r="C4" s="2">
         <v>2172</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4" s="2">
         <v>201.56215469613261</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4" s="2">
         <v>1109</v>
       </c>
-      <c r="E4" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F4" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="9"/>
+      <c r="C5" s="2">
         <v>3021</v>
       </c>
-      <c r="C5" s="2">
+      <c r="D5" s="2">
         <v>219.91029460443562</v>
       </c>
-      <c r="D5" s="2">
+      <c r="E5" s="2">
         <v>1331</v>
       </c>
-      <c r="E5" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F5" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="2">
+        <v>21</v>
+      </c>
+      <c r="B6" s="9"/>
+      <c r="C6" s="2">
         <v>1130</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D6" s="2">
         <v>162.64601769911505</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="2">
         <v>789</v>
       </c>
-      <c r="E6" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F6" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="9"/>
+      <c r="C7" s="2">
         <v>3670</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7" s="2">
         <v>216.36730245231607</v>
       </c>
-      <c r="D7" s="2">
+      <c r="E7" s="2">
         <v>38833</v>
       </c>
-      <c r="E7" s="2">
-        <v>75</v>
-      </c>
-      <c r="F7" s="8">
+      <c r="F7" s="2">
+        <v>75</v>
+      </c>
+      <c r="G7" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="2">
+        <v>2934</v>
+      </c>
+      <c r="D8" s="2">
+        <v>220.69904567143831</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1686</v>
+      </c>
+      <c r="F8" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2">
-        <v>2934</v>
-      </c>
-      <c r="C8" s="2">
-        <v>220.69904567143831</v>
-      </c>
-      <c r="D8" s="2">
-        <v>1686</v>
-      </c>
-      <c r="E8" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="2">
+        <v>3086</v>
+      </c>
+      <c r="D9" s="2">
+        <v>208.0758263123785</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1225</v>
+      </c>
+      <c r="F9" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="2">
+        <v>152</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2958.2434210526317</v>
+      </c>
+      <c r="E10" s="2">
+        <v>229613</v>
+      </c>
+      <c r="F10" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="2">
-        <v>3086</v>
-      </c>
-      <c r="C9" s="2">
-        <v>208.0758263123785</v>
-      </c>
-      <c r="D9" s="2">
-        <v>1225</v>
-      </c>
-      <c r="E9" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="B11" s="9"/>
+      <c r="C11" s="2">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2">
+        <v>53051.666666666664</v>
+      </c>
+      <c r="E11" s="2">
+        <v>635166</v>
+      </c>
+      <c r="F11" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="2">
+        <v>377</v>
+      </c>
+      <c r="D12" s="2">
+        <v>200.51989389920425</v>
+      </c>
+      <c r="E12" s="2">
+        <v>2208</v>
+      </c>
+      <c r="F12" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="2">
+        <v>364</v>
+      </c>
+      <c r="D13" s="2">
+        <v>163.33791208791209</v>
+      </c>
+      <c r="E13" s="2">
+        <v>863</v>
+      </c>
+      <c r="F13" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2">
-        <v>152</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2958.2434210526317</v>
-      </c>
-      <c r="D10" s="2">
-        <v>229613</v>
-      </c>
-      <c r="E10" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="B14" s="9"/>
+      <c r="C14" s="2">
+        <v>181</v>
+      </c>
+      <c r="D14" s="2">
+        <v>377.8011049723757</v>
+      </c>
+      <c r="E14" s="2">
+        <v>2853</v>
+      </c>
+      <c r="F14" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B15" s="9"/>
+      <c r="C15" s="2">
+        <v>151</v>
+      </c>
+      <c r="D15" s="2">
+        <v>881.42384105960264</v>
+      </c>
+      <c r="E15" s="2">
+        <v>10948</v>
+      </c>
+      <c r="F15" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="2">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="2">
-        <v>53051.666666666664</v>
-      </c>
-      <c r="D11" s="2">
-        <v>635166</v>
-      </c>
-      <c r="E11" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="2">
-        <v>377</v>
-      </c>
-      <c r="C12" s="2">
-        <v>200.51989389920425</v>
-      </c>
-      <c r="D12" s="2">
-        <v>2208</v>
-      </c>
-      <c r="E12" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="2">
-        <v>364</v>
-      </c>
-      <c r="C13" s="2">
-        <v>163.33791208791209</v>
-      </c>
-      <c r="D13" s="2">
-        <v>863</v>
-      </c>
-      <c r="E13" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2">
-        <v>181</v>
-      </c>
-      <c r="C14" s="2">
-        <v>377.8011049723757</v>
-      </c>
-      <c r="D14" s="2">
-        <v>2853</v>
-      </c>
-      <c r="E14" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2">
-        <v>151</v>
-      </c>
-      <c r="C15" s="2">
-        <v>881.42384105960264</v>
-      </c>
-      <c r="D15" s="2">
-        <v>10948</v>
-      </c>
-      <c r="E15" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="2">
+      <c r="B17" s="9"/>
+      <c r="C17" s="2">
+        <v>2</v>
+      </c>
+      <c r="D17" s="6">
+        <v>490</v>
+      </c>
+      <c r="E17" s="6">
+        <v>650</v>
+      </c>
+      <c r="F17" s="6">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="2">
         <v>0</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="2">
-        <v>2</v>
-      </c>
-      <c r="C17" s="6">
-        <v>490</v>
-      </c>
-      <c r="D17" s="6">
-        <v>650</v>
-      </c>
-      <c r="E17" s="6">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+      <c r="D18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="2">
-        <v>0</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="2">
-        <v>0</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B23" s="7"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>